<commit_message>
📊 Update places Excel
</commit_message>
<xml_diff>
--- a/places.xlsx
+++ b/places.xlsx
@@ -8,6 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="📋 All Places" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📍 Fort Lauderdale" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📍 Sunrise" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,12 +43,26 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="001A1A2E"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000066CC"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="00888888"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +82,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0016213E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -100,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -111,11 +137,26 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -587,15 +628,306 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
+          <t>[Fort Lauderdale] WhatSub Sub Shop</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Sandwiches/Subs</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?q=WhatSub+Sub+Shop+Fort+Lauderdale+FL</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>A sub sandwich shop located in Fort Lauderdale, Florida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>[Sunrise] TEN TEN Chinese Seafood Dim Sum Restaurant</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Chinese Dim Sum, Seafood</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Opens at 11:00 AM</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?q=TEN+TEN+Chinese+Seafood+Dim+Sum+Restaurant+Sunrise+FL</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Authentic Chinese dim sum restaurant in Broward County offering fresh, affordable food in a welcoming atmosphere. Recommended for lunch for the ultimate dim sum experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>🎯  ACTIVITIES &amp; ATTRACTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Price Range</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
           <t>No entries yet</t>
         </is>
       </c>
     </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A7:M7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>📍  FORT LAUDERDALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>🍽️  RESTAURANTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Cuisine</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Price Range</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Online Ordering</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>WhatSub Sub Shop</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Sandwiches/Subs</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?q=WhatSub+Sub+Shop+Fort+Lauderdale+FL</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>A sub sandwich shop located in Fort Lauderdale, Florida.</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>🎯  ACTIVITIES &amp; ATTRACTIONS</t>
         </is>
@@ -604,84 +936,309 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>Categories</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Price Range</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>No entries yet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>📍  SUNRISE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>🍽️  RESTAURANTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Cuisine</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Price Range</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Online Ordering</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TEN TEN Chinese Seafood Dim Sum Restaurant</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Chinese Dim Sum, Seafood</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Opens at 11:00 AM</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>https://maps.google.com/?q=TEN+TEN+Chinese+Seafood+Dim+Sum+Restaurant+Sunrise+FL</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Authentic Chinese dim sum restaurant in Broward County offering fresh, affordable food in a welcoming atmosphere. Recommended for lunch for the ultimate dim sum experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>🎯  ACTIVITIES &amp; ATTRACTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Categories</t>
+        </is>
+      </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Categories</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Phone</t>
+          <t>Hours</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Hours</t>
+          <t>Price Range</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Price Range</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Google Maps</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Book Online</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Book Online</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>No entries yet</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A8:M8"/>
-    <mergeCell ref="A6:M6"/>
-    <mergeCell ref="A2:N2"/>
+  <mergeCells count="4">
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>